<commit_message>
fix(ttb): move recipient phone box from header to bottom under Received By column
</commit_message>
<xml_diff>
--- a/Data_Crew_Kapal_PT_CPL_2026_Clean.xlsx
+++ b/Data_Crew_Kapal_PT_CPL_2026_Clean.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Dashboard-cpg web\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85CE2018-5FE3-4A9E-9F97-0FE38AE8CF7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDB3D3B9-BA3D-46A4-A13B-95E04984CCF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11691" uniqueCount="3059">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11715" uniqueCount="3066">
   <si>
     <t>PT. CINDARA PRATAMA LINES</t>
   </si>
@@ -9212,6 +9212,27 @@
   </si>
   <si>
     <t>SPOB RR 3001</t>
+  </si>
+  <si>
+    <t>LXI</t>
+  </si>
+  <si>
+    <t>GAJ</t>
+  </si>
+  <si>
+    <t>Ardiyan</t>
+  </si>
+  <si>
+    <t>Mulyadi</t>
+  </si>
+  <si>
+    <t>Fadli Babe</t>
+  </si>
+  <si>
+    <t>Doni</t>
+  </si>
+  <si>
+    <t>Staf Logistik</t>
   </si>
 </sst>
 </file>
@@ -9403,7 +9424,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -9441,11 +9462,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFCBD5E1"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFCBD5E1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -9523,6 +9555,15 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="16" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -9533,14 +9574,14 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -9898,23 +9939,23 @@
       <c r="K6" s="30"/>
     </row>
     <row r="7" spans="2:14" ht="23.25" x14ac:dyDescent="0.25">
-      <c r="B7" s="34">
+      <c r="B7" s="37">
         <v>60</v>
       </c>
       <c r="C7" s="30"/>
-      <c r="D7" s="33">
+      <c r="D7" s="36">
         <v>633</v>
       </c>
       <c r="E7" s="30"/>
-      <c r="F7" s="37">
+      <c r="F7" s="33">
         <v>531</v>
       </c>
       <c r="G7" s="30"/>
-      <c r="H7" s="35">
+      <c r="H7" s="31">
         <v>70</v>
       </c>
       <c r="I7" s="30"/>
-      <c r="J7" s="36">
+      <c r="J7" s="32">
         <v>32</v>
       </c>
       <c r="K7" s="30"/>
@@ -12346,16 +12387,16 @@
       </c>
     </row>
     <row r="72" spans="2:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B72" s="31" t="s">
+      <c r="B72" s="34" t="s">
         <v>258</v>
       </c>
-      <c r="C72" s="32"/>
-      <c r="D72" s="32"/>
-      <c r="E72" s="32"/>
-      <c r="F72" s="32"/>
-      <c r="G72" s="32"/>
-      <c r="H72" s="32"/>
-      <c r="I72" s="32"/>
+      <c r="C72" s="35"/>
+      <c r="D72" s="35"/>
+      <c r="E72" s="35"/>
+      <c r="F72" s="35"/>
+      <c r="G72" s="35"/>
+      <c r="H72" s="35"/>
+      <c r="I72" s="35"/>
       <c r="J72" s="15">
         <f>SUM(J12:J71)</f>
         <v>632</v>
@@ -12379,17 +12420,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="J6:K6"/>
-    <mergeCell ref="H7:I7"/>
-    <mergeCell ref="J7:K7"/>
-    <mergeCell ref="F6:G6"/>
-    <mergeCell ref="F7:G7"/>
     <mergeCell ref="D6:E6"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B72:I72"/>
     <mergeCell ref="D7:E7"/>
     <mergeCell ref="B7:C7"/>
     <mergeCell ref="H6:I6"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="H7:I7"/>
+    <mergeCell ref="J7:K7"/>
+    <mergeCell ref="F6:G6"/>
+    <mergeCell ref="F7:G7"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -12397,7 +12438,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:R637"/>
+  <dimension ref="A1:R641"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11" customWidth="1"/>
@@ -47903,6 +47944,110 @@
       </c>
       <c r="R637" s="17" t="s">
         <v>73</v>
+      </c>
+    </row>
+    <row r="638" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A638" s="6">
+        <v>634</v>
+      </c>
+      <c r="B638" s="38" t="s">
+        <v>3059</v>
+      </c>
+      <c r="C638" s="39" t="s">
+        <v>3060</v>
+      </c>
+      <c r="D638" s="38" t="s">
+        <v>257</v>
+      </c>
+      <c r="E638" s="38">
+        <v>1</v>
+      </c>
+      <c r="G638" s="39" t="s">
+        <v>3061</v>
+      </c>
+      <c r="H638" s="40" t="s">
+        <v>3065</v>
+      </c>
+      <c r="K638" s="9" t="s">
+        <v>2905</v>
+      </c>
+    </row>
+    <row r="639" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A639" s="6">
+        <v>635</v>
+      </c>
+      <c r="B639" s="38" t="s">
+        <v>3059</v>
+      </c>
+      <c r="C639" s="39" t="s">
+        <v>3060</v>
+      </c>
+      <c r="D639" s="38" t="s">
+        <v>257</v>
+      </c>
+      <c r="E639" s="38">
+        <v>2</v>
+      </c>
+      <c r="G639" s="39" t="s">
+        <v>3062</v>
+      </c>
+      <c r="H639" s="40" t="s">
+        <v>3065</v>
+      </c>
+      <c r="K639" s="6" t="s">
+        <v>2914</v>
+      </c>
+    </row>
+    <row r="640" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A640" s="6">
+        <v>636</v>
+      </c>
+      <c r="B640" s="38" t="s">
+        <v>3059</v>
+      </c>
+      <c r="C640" s="39" t="s">
+        <v>3060</v>
+      </c>
+      <c r="D640" s="38" t="s">
+        <v>257</v>
+      </c>
+      <c r="E640" s="38">
+        <v>3</v>
+      </c>
+      <c r="G640" s="39" t="s">
+        <v>3063</v>
+      </c>
+      <c r="H640" s="40" t="s">
+        <v>3065</v>
+      </c>
+      <c r="K640" s="9" t="s">
+        <v>2891</v>
+      </c>
+    </row>
+    <row r="641" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A641" s="6">
+        <v>637</v>
+      </c>
+      <c r="B641" s="38" t="s">
+        <v>3059</v>
+      </c>
+      <c r="C641" s="39" t="s">
+        <v>3060</v>
+      </c>
+      <c r="D641" s="38" t="s">
+        <v>257</v>
+      </c>
+      <c r="E641" s="38">
+        <v>4</v>
+      </c>
+      <c r="G641" s="39" t="s">
+        <v>3064</v>
+      </c>
+      <c r="H641" s="40" t="s">
+        <v>3065</v>
+      </c>
+      <c r="K641" s="9" t="s">
+        <v>2922</v>
       </c>
     </row>
   </sheetData>

</xml_diff>